<commit_message>
Run natively on Windows with PowerShell and a local PostgreSQL
The Makefile needs make and bash, and `make up` needs docker or
`su postgres`. scripts/windows.ps1 runs the same python -m src.* steps
in the same order; scripts/windows_init_db.sql does the one-time role,
database and grant setup that db_up.sh does on native Linux. Also:
make_workbook used a hard-coded python3 (absent on Windows), and
.gitattributes keeps the .asc extracts byte-identical across OSes.
The setup workbook gains a Windows native tab. Docker/WSL paths unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165Za6gtPggDtMyRg2Z7ePj
</commit_message>
<xml_diff>
--- a/deliverables/Setup_Workbook.xlsx
+++ b/deliverables/Setup_Workbook.xlsx
@@ -13,9 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Build" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Open the site" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Use it" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Troubleshooting" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every command" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Windows native" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Troubleshooting" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reset" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every command" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -562,7 +563,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="51" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Works on</t>
@@ -570,7 +571,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Windows with WSL2 (recommended), macOS, or Linux. Native Windows without WSL is not supported: the build uses make and bash.</t>
+          <t>Windows with WSL2, macOS, or Linux (tabs 1-4). Native Windows without WSL or Docker, using a locally installed PostgreSQL and PowerShell: see the “Windows native” tab instead of tabs 1-4.</t>
         </is>
       </c>
     </row>
@@ -610,7 +611,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
+    <row r="9" ht="51" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Where to type commands</t>
@@ -618,7 +619,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>On Windows: the Ubuntu app (WSL), NOT PowerShell. Type  wsl  in the Start menu if you do not see it. Every command in this workbook is for that terminal.</t>
+          <t>WSL route: the Ubuntu app, not PowerShell. Every command in tabs 1-5 is for that terminal. Native route: PowerShell (or the VS Code terminal), commands in the “Windows native” tab only.</t>
         </is>
       </c>
     </row>
@@ -654,7 +655,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>1 Install  →  2 Get the code  →  3 Build  →  4 Open the site  →  5 Use it  →  Troubleshooting  →  Reset  →  Every command</t>
+          <t>1 Install  →  2 Get the code  →  3 Build  →  4 Open the site  →  5 Use it  →  Windows native  →  Troubleshooting  →  Reset  →  Every command</t>
         </is>
       </c>
     </row>
@@ -673,6 +674,266 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Every command, in order, with nothing else</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>For when you have done this once and just want to paste. Lines starting # are comments, not commands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Command</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="10" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t># First time only</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>sudo apt update &amp;&amp; sudo apt install -y make git python3-venv python3-pip</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Windows: in the Ubuntu app, with Docker Desktop running</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>cd ~ &amp;&amp; git clone https://github.com/robindebruyne1234/Loan-valid-DQ.git</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Not in /mnt/c</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>cd Loan-valid-DQ &amp;&amp; git checkout ccr-46f6f45a-t9wtd4</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>python3 -m venv .venv</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>source .venv/bin/activate</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Repeat in every new terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>make deps</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>make up</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Starts PostgreSQL in Docker</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>make build</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>About 6 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>make web-open</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Opens http://localhost:8080</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t># Every time after that</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>cd ~/Loan-valid-DQ &amp;&amp; source .venv/bin/activate &amp;&amp; make up &amp;&amp; make web-open</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t># Optional extras</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>make demo-login</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>The privacy walkthrough in the terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>make demo-interactive</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Pick a person, type the code, run your own SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>make test</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Run the tests</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1790,6 +2051,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Windows without WSL or Docker</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>PowerShell in the repository folder (VS Code: Terminal → New Terminal). Uses your own PostgreSQL. Replaces tabs 1-4; tab 5 is the same.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>What you are doing</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Command (copy this cell)</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>You should see</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>If you do not</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Check Python is 3.11 or newer.</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>py -3 --version</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Python 3.11.x or newer.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Not found or older: install Python 3.11+ from python.org (tick “Add to PATH”).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="51" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr"/>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Check PostgreSQL is installed and running (Services → postgresql-x64-16).</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Get-Service postgresql*</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Status Running.</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Not listed: install PostgreSQL 16 from postgresql.org (EDB installer). Stopped: Start-Service postgresql-x64-16 (as administrator).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Allow this script to run in this window only.</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Set-ExecutionPolicy -Scope Process Bypass</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>No output.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Or prefix every command with: powershell -ExecutionPolicy Bypass -File</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="51" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Create .venv and install the Python packages.</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>scripts\windows.ps1 setup</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>setup | dependencies installed into .venv</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>“needs 3.11 or newer”: pass your interpreter, e.g.  scripts\windows.ps1 setup -Python C:\Python312\python.exe</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="68" customHeight="1">
+      <c r="A9" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Create the project role and database (once). psql asks for the password you chose for the postgres superuser when installing PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>scripts\windows.ps1 init-db</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>CREATE ROLE, CREATE DATABASE, GRANT … then init-db | done</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>“psql.exe not found”: add C:\Program Files\PostgreSQL\16\bin to PATH. “password authentication failed for user postgres”: wrong superuser password.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="85" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr"/>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Build everything (same steps as make build, without the LLM).</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>scripts\windows.ps1 build</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Ends with “241 passed” and build | done.</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>“Cannot connect to PostgreSQL”: service stopped, or init-db not run. A PGUSER/PGPASSWORD set for another login overrides the project defaults: Remove-Item Env:PGUSER, Env:PGPASSWORD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Open the walkthrough in your browser. Then follow tab 5.</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>scripts\windows.ps1 web-open</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>serving the walkthrough on http://localhost:8080, and a browser tab opens.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Port in use:  scripts\windows.ps1 web-open -WebPort 8081</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr"/>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Later: tests only, or the stakeholder console demo.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>scripts\windows.ps1 test
+scripts\windows.ps1 demo-login</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>“241 passed”; the console demo ends with === END ===.</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Run build first if the database was reset.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"yes,no"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2151,7 +2698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2305,264 +2852,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:C20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="64" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Every command, in order, with nothing else</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>For when you have done this once and just want to paste. Lines starting # are comments, not commands.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Command</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t># First time only</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>sudo apt update &amp;&amp; sudo apt install -y make git python3-venv python3-pip</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Windows: in the Ubuntu app, with Docker Desktop running</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>cd ~ &amp;&amp; git clone https://github.com/robindebruyne1234/Loan-valid-DQ.git</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Not in /mnt/c</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>cd Loan-valid-DQ &amp;&amp; git checkout ccr-46f6f45a-t9wtd4</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>python3 -m venv .venv</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>source .venv/bin/activate</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Repeat in every new terminal</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>make deps</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>make up</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Starts PostgreSQL in Docker</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>make build</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>About 6 minutes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>make web-open</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Opens http://localhost:8080</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t># Every time after that</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>cd ~/Loan-valid-DQ &amp;&amp; source .venv/bin/activate &amp;&amp; make up &amp;&amp; make web-open</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="10" t="inlineStr"/>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t># Optional extras</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>make demo-login</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>The privacy walkthrough in the terminal</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>make demo-interactive</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Pick a person, type the code, run your own SQL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>make test</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Run the tests</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>